<commit_message>
feat: add user import template spreadsheet for bulk data uploads
</commit_message>
<xml_diff>
--- a/public/template/user_import_template.xlsx
+++ b/public/template/user_import_template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,117 +439,122 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>positionName</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>roleName</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>groupName</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>phoneNumber</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>gender</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>dateOfBirth</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>maritalStatus</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>citizenIdNumber</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>citizenIdIssueDate</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>citizenIdIssuePlace</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>currentAddress</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>currentCity</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>placeOfBirth</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>placeOfOrigin</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>nationality</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>ethnicity</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>religion</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>permanentAddress</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>permanentCity</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>bankAccountNumber</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>bankAccountName</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>bankName</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>bankBranch</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>roleName</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement user attendance tracking page with monthly summary and request details view
</commit_message>
<xml_diff>
--- a/public/template/user_import_template.xlsx
+++ b/public/template/user_import_template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AC1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,125 +434,130 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>englishName</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>departmentName</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>positionName</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>roleName</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>jobTitleName</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>groupName</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>phoneNumber</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>gender</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>dateOfBirth</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>maritalStatus</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>citizenIdNumber</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>citizenIdIssueDate</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>citizenIdIssuePlace</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>currentAddress</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>currentCity</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>placeOfBirth</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>placeOfOrigin</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>nationality</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>ethnicity</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>religion</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>permanentAddress</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>permanentCity</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>bankAccountNumber</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>bankAccountName</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>bankName</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>bankBranch</t>
         </is>

</xml_diff>